<commit_message>
Add different ggv plot views and fix magic formula parameters.
</commit_message>
<xml_diff>
--- a/Vehicles/F24_Continuous_Torque/parameters.xlsx
+++ b/Vehicles/F24_Continuous_Torque/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ryan Koo\PycharmProjects\Steady-State Lap Time Simulator\Vehicles\F24_Continuous_Torque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A40013FE-B15C-4EDB-A123-8D617D6EB9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5103CD-93D6-4C9D-A0C8-CABF7BD57F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{DAA64B5D-7408-4506-8E44-C0800644134F}"/>
   </bookViews>
@@ -897,7 +897,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="1">
-        <v>0.1404</v>
+        <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>4</v>

</xml_diff>